<commit_message>
fix BM dung sx
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/template_NhatKy_SanXuat.xlsx
+++ b/Data_Product/App_Data/template_NhatKy_SanXuat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software\ThongKePKH\DATAPRODUCT_DEV\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CAE96F3-814B-4DF3-991B-8A9573CC5974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66F43D2-C84E-4EF9-BFD9-E3A8166FD783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{9F82862B-75F6-4CCB-A11A-BFD2F7A1C8D2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="31">
   <si>
     <t>STT</t>
   </si>
@@ -143,6 +143,9 @@
   </si>
   <si>
     <t>Cụm Thêm 1</t>
+  </si>
+  <si>
+    <t>Thời gian dừng</t>
   </si>
 </sst>
 </file>
@@ -370,7 +373,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -427,6 +430,9 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -450,6 +456,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -973,155 +985,164 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84BEA158-B0A7-4F33-BECC-35D22A70C1E6}">
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="17" style="1" customWidth="1"/>
     <col min="4" max="5" width="21.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.42578125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="9" style="1" customWidth="1"/>
-    <col min="11" max="16" width="9.140625" style="1"/>
-    <col min="17" max="17" width="10.85546875" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="12.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9" style="1" customWidth="1"/>
+    <col min="12" max="17" width="9.140625" style="1"/>
+    <col min="18" max="18" width="10.85546875" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="6"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
       <c r="H1" s="6"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="8"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="8"/>
     </row>
-    <row r="2" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="9"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="10"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="5"/>
       <c r="H2" s="10"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="12"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="12"/>
     </row>
-    <row r="3" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="9"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="13"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="5"/>
       <c r="H3" s="13"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="14"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="14"/>
     </row>
-    <row r="4" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+    <row r="4" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
     </row>
-    <row r="5" spans="1:18" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+    <row r="5" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="H6" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="26" t="s">
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="27"/>
-      <c r="M6" s="24" t="s">
+      <c r="M6" s="28"/>
+      <c r="N6" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="24" t="s">
+      <c r="O6" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="24" t="s">
+      <c r="P6" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="P6" s="28" t="s">
+      <c r="Q6" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" s="24" t="s">
+      <c r="R6" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="R6" s="24" t="s">
+      <c r="S6" s="25" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:18" s="16" customFormat="1" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="19" t="s">
+    <row r="7" spans="1:19" s="16" customFormat="1" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="26"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="I7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="J7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="K7" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="K7" s="20" t="s">
+      <c r="L7" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="L7" s="21" t="s">
+      <c r="M7" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="29"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="25"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="30"/>
+      <c r="R7" s="26"/>
+      <c r="S7" s="26"/>
     </row>
-    <row r="8" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>2</v>
       </c>
@@ -1137,38 +1158,42 @@
       <c r="E8" s="17">
         <v>0.70833333333333337</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="24">
+        <f>(E8-D8)*24*60</f>
+        <v>570</v>
+      </c>
+      <c r="G8" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="2">
         <v>1</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="2">
         <v>2.5</v>
       </c>
-      <c r="I8" s="15">
+      <c r="J8" s="15">
         <v>3.5</v>
       </c>
-      <c r="J8" s="15">
-        <f>H8+I8</f>
+      <c r="K8" s="15">
+        <f>I8+J8</f>
         <v>6</v>
       </c>
-      <c r="K8" s="15" t="s">
+      <c r="L8" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="L8" s="15"/>
       <c r="M8" s="15"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
-      <c r="P8" s="15">
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q8" s="15" t="s">
+      <c r="R8" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R8" s="15"/>
+      <c r="S8" s="15"/>
     </row>
-    <row r="9" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>3</v>
       </c>
@@ -1184,32 +1209,36 @@
       <c r="E9" s="17">
         <v>0.75</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="24">
+        <f t="shared" ref="F9:F15" si="0">(E9-D9)*24*60</f>
+        <v>569.99999999999943</v>
+      </c>
+      <c r="G9" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15">
-        <f t="shared" ref="J9:J15" si="0">H9+I9</f>
+      <c r="I9" s="2"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15">
+        <f t="shared" ref="K9:K15" si="1">I9+J9</f>
         <v>0</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15" t="s">
+      <c r="L9" s="15"/>
+      <c r="M9" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="M9" s="15"/>
       <c r="N9" s="15"/>
       <c r="O9" s="15"/>
-      <c r="P9" s="15">
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q9" s="15" t="s">
+      <c r="R9" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
     </row>
-    <row r="10" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>4</v>
       </c>
@@ -1225,32 +1254,36 @@
       <c r="E10" s="17">
         <v>0.79166666666666696</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="24">
+        <f t="shared" si="0"/>
+        <v>570.00000000000091</v>
+      </c>
+      <c r="G10" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15">
-        <f t="shared" si="0"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K10" s="15"/>
       <c r="L10" s="15"/>
-      <c r="M10" s="15" t="s">
+      <c r="M10" s="15"/>
+      <c r="N10" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="N10" s="15"/>
       <c r="O10" s="15"/>
-      <c r="P10" s="15">
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q10" s="15" t="s">
+      <c r="R10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
     </row>
-    <row r="11" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>5</v>
       </c>
@@ -1266,32 +1299,36 @@
       <c r="E11" s="17">
         <v>0.83333333333333304</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="24">
+        <f t="shared" si="0"/>
+        <v>569.99999999999955</v>
+      </c>
+      <c r="G11" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15">
-        <f t="shared" si="0"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K11" s="15"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
-      <c r="N11" s="15" t="s">
+      <c r="N11" s="15"/>
+      <c r="O11" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15">
+      <c r="P11" s="15"/>
+      <c r="Q11" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q11" s="15" t="s">
+      <c r="R11" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="R11" s="15"/>
+      <c r="S11" s="15"/>
     </row>
-    <row r="12" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>6</v>
       </c>
@@ -1307,32 +1344,36 @@
       <c r="E12" s="17">
         <v>0.875</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="24">
+        <f t="shared" si="0"/>
+        <v>569.99999999999943</v>
+      </c>
+      <c r="G12" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15">
-        <f t="shared" si="0"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K12" s="15"/>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
       <c r="N12" s="15"/>
-      <c r="O12" s="15" t="s">
+      <c r="O12" s="15"/>
+      <c r="P12" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="P12" s="15">
+      <c r="Q12" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q12" s="15" t="s">
+      <c r="R12" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
     </row>
-    <row r="13" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>7</v>
       </c>
@@ -1348,30 +1389,34 @@
       <c r="E13" s="17">
         <v>0.91666666666666696</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="24">
+        <f t="shared" si="0"/>
+        <v>570.00000000000091</v>
+      </c>
+      <c r="G13" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15">
-        <f t="shared" si="0"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K13" s="15"/>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
       <c r="N13" s="15"/>
       <c r="O13" s="15"/>
-      <c r="P13" s="15">
+      <c r="P13" s="15"/>
+      <c r="Q13" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q13" s="15" t="s">
+      <c r="R13" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="R13" s="15"/>
+      <c r="S13" s="15"/>
     </row>
-    <row r="14" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>8</v>
       </c>
@@ -1387,30 +1432,34 @@
       <c r="E14" s="17">
         <v>0.95833333333333304</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="24">
+        <f t="shared" si="0"/>
+        <v>569.99999999999955</v>
+      </c>
+      <c r="G14" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15">
-        <f t="shared" si="0"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K14" s="15"/>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
       <c r="N14" s="15"/>
       <c r="O14" s="15"/>
-      <c r="P14" s="15">
+      <c r="P14" s="15"/>
+      <c r="Q14" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q14" s="15" t="s">
+      <c r="R14" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
     </row>
-    <row r="15" spans="1:18" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" s="16" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>9</v>
       </c>
@@ -1426,46 +1475,51 @@
       <c r="E15" s="17">
         <v>1</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="24">
+        <f t="shared" si="0"/>
+        <v>569.99999999999955</v>
+      </c>
+      <c r="G15" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15">
-        <f t="shared" si="0"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K15" s="15"/>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
       <c r="N15" s="15"/>
       <c r="O15" s="15"/>
-      <c r="P15" s="15">
+      <c r="P15" s="15"/>
+      <c r="Q15" s="15">
         <v>2.5</v>
       </c>
-      <c r="Q15" s="15" t="s">
+      <c r="R15" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="R15" s="15"/>
+      <c r="S15" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A4:J4"/>
+  <mergeCells count="16">
+    <mergeCell ref="A4:K4"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:K6"/>
     <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="Q6:Q7"/>
     <mergeCell ref="R6:R7"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="S6:S7"/>
+    <mergeCell ref="L6:M6"/>
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="O6:O7"/>
     <mergeCell ref="P6:P7"/>
+    <mergeCell ref="Q6:Q7"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.43" right="0.34" top="0.31" bottom="0.28000000000000003" header="0.3" footer="0.3"/>

</xml_diff>